<commit_message>
Bulls: add Elite Reads article URLs to launch sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P8umMQtAY5S5sHQF7eLKEP
</commit_message>
<xml_diff>
--- a/bulls/lists/2026-10-05_bulls_launch/Bulls_3_offers_2026-10-05.xlsx
+++ b/bulls/lists/2026-10-05_bulls_launch/Bulls_3_offers_2026-10-05.xlsx
@@ -630,11 +630,6 @@
     <author>Claude</author>
   </authors>
   <commentList>
-    <comment ref="E2" authorId="0" shapeId="0">
-      <text>
-        <t>Pending: Elite Reads article is being written. Add the article URL when published.</t>
-      </text>
-    </comment>
     <comment ref="G2" authorId="0" shapeId="0">
       <text>
         <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
@@ -650,19 +645,9 @@
     <author>Claude</author>
   </authors>
   <commentList>
-    <comment ref="E2" authorId="0" shapeId="0">
-      <text>
-        <t>Pending: Elite Reads article is being written. Add the article URL when published.</t>
-      </text>
-    </comment>
     <comment ref="G2" authorId="0" shapeId="0">
       <text>
         <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
-      </text>
-    </comment>
-    <comment ref="E3" authorId="0" shapeId="0">
-      <text>
-        <t>Pending: Elite Reads article is being written. Add the article URL when published.</t>
       </text>
     </comment>
     <comment ref="G3" authorId="0" shapeId="0">
@@ -1059,7 +1044,11 @@
           <t>https://quxfjrw.com/adServe/aff?cmpid=703649&amp;pid=458124&amp;ap1=458124&amp;dp1=458124&amp;dp2=elite-reads.com&amp;dlink=https%3A%2F%2Fwww.ncl.com</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/norwegian-cruise-line-ships-guide/</t>
+        </is>
+      </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Intango</t>
@@ -1143,7 +1132,11 @@
           <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fwww.waipu.tv&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/waipu-tv-german-tv-streaming/</t>
+        </is>
+      </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
           <t>digidip</t>
@@ -1154,25 +1147,29 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
+          <t>Sky Deutschland</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
           <t>sky.de</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>sky.de</t>
-        </is>
-      </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
           <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fwww.sky.de&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/sky-deutschland-packages-worth-it/</t>
+        </is>
+      </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
           <t>digidip</t>

</xml_diff>

<commit_message>
Bulls: launch sheet in one tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P8umMQtAY5S5sHQF7eLKEP
</commit_message>
<xml_diff>
--- a/bulls/lists/2026-10-05_bulls_launch/Bulls_3_offers_2026-10-05.xlsx
+++ b/bulls/lists/2026-10-05_bulls_launch/Bulls_3_offers_2026-10-05.xlsx
@@ -6,8 +6,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2300" yWindow="2320" windowWidth="26840" windowHeight="15940" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026-10-05_Intango" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2026-10-05_digidip" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-10-05" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -635,22 +634,12 @@
         <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
       </text>
     </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Claude</author>
-  </authors>
-  <commentList>
-    <comment ref="G2" authorId="0" shapeId="0">
+    <comment ref="G3" authorId="0" shapeId="0">
       <text>
         <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
       </text>
     </comment>
-    <comment ref="G3" authorId="0" shapeId="0">
+    <comment ref="G4" authorId="0" shapeId="0">
       <text>
         <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
       </text>
@@ -980,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -1056,126 +1045,71 @@
       </c>
       <c r="G2" s="2" t="n"/>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col width="60" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Geos</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Pure domain</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Offer link</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Blog url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Affiliate Network</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Service Credential Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>waipu.tv</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>waipu.tv</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fwww.waipu.tv&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>https://www.elite-reads.com/waipu-tv-german-tv-streaming/</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>digidip</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-    </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
+          <t>waipu.tv</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>waipu.tv</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fwww.waipu.tv&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/waipu-tv-german-tv-streaming/</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>digidip</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
           <t>Sky Deutschland</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>sky.de</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fwww.sky.de&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>https://www.elite-reads.com/sky-deutschland-packages-worth-it/</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>digidip</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Bulls: fill Service Credential Name per network
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P8umMQtAY5S5sHQF7eLKEP
</commit_message>
<xml_diff>
--- a/bulls/lists/2026-10-05_bulls_launch/Bulls_3_offers_2026-10-05.xlsx
+++ b/bulls/lists/2026-10-05_bulls_launch/Bulls_3_offers_2026-10-05.xlsx
@@ -621,31 +621,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Claude</author>
-  </authors>
-  <commentList>
-    <comment ref="G2" authorId="0" shapeId="0">
-      <text>
-        <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
-      </text>
-    </comment>
-    <comment ref="G3" authorId="0" shapeId="0">
-      <text>
-        <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
-      </text>
-    </comment>
-    <comment ref="G4" authorId="0" shapeId="0">
-      <text>
-        <t>Pending: Service Credential Name not provided yet (example format: 'NYJL - CJ - RDV - NY').</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1043,7 +1018,11 @@
           <t>Intango</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>NYJL - Intango - RDV - NY</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1076,7 +1055,11 @@
           <t>digidip</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>NYJL - digidip - RDV - NY</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1109,10 +1092,13 @@
           <t>digidip</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>NYJL - digidip - RDV - NY</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>